<commit_message>
Upload traffic plan folder
</commit_message>
<xml_diff>
--- a/Mạng lưới/outputs/ket_qua_toi_uu_mang_luoi.xlsx
+++ b/Mạng lưới/outputs/ket_qua_toi_uu_mang_luoi.xlsx
@@ -557,46 +557,46 @@
         <v>50</v>
       </c>
       <c r="G2" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="H2" t="n">
         <v>34</v>
       </c>
       <c r="I2" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="L2" t="n">
-        <v>802.5131018603657</v>
+        <v>1147.915106176677</v>
       </c>
       <c r="M2" t="n">
-        <v>796.792389317889</v>
+        <v>1123.759506613288</v>
       </c>
       <c r="N2" t="n">
-        <v>0.712849737806782</v>
+        <v>2.104301915134094</v>
       </c>
       <c r="O2" t="n">
-        <v>355.7201256776642</v>
+        <v>337.8839538197327</v>
       </c>
       <c r="P2" t="n">
-        <v>363.5817245475808</v>
+        <v>359.4645859889835</v>
       </c>
       <c r="Q2" t="n">
-        <v>-2.210051752045208</v>
+        <v>-6.386995276125012</v>
       </c>
       <c r="R2" t="n">
         <v>29652.72512726851</v>
       </c>
       <c r="S2" t="n">
-        <v>24200.12364833376</v>
+        <v>23681.3051851498</v>
       </c>
       <c r="T2" t="n">
-        <v>18.38819688757901</v>
+        <v>20.13784539697303</v>
       </c>
       <c r="U2" t="n">
         <v>150</v>
@@ -624,46 +624,46 @@
         <v>49</v>
       </c>
       <c r="G3" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H3" t="n">
         <v>35</v>
       </c>
       <c r="I3" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J3" t="n">
         <v>25</v>
       </c>
       <c r="K3" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="L3" t="n">
-        <v>277.0707107198699</v>
+        <v>277.1742180323049</v>
       </c>
       <c r="M3" t="n">
-        <v>277.0306914955323</v>
+        <v>277.0678421476935</v>
       </c>
       <c r="N3" t="n">
-        <v>0.01444368631879753</v>
+        <v>0.0383787082963613</v>
       </c>
       <c r="O3" t="n">
-        <v>14.54821163182095</v>
+        <v>7.835458585034194</v>
       </c>
       <c r="P3" t="n">
-        <v>13.26177195317458</v>
+        <v>7.716024500709814</v>
       </c>
       <c r="Q3" t="n">
-        <v>8.842596679254854</v>
+        <v>1.524276888560176</v>
       </c>
       <c r="R3" t="n">
         <v>1529.994475441986</v>
       </c>
       <c r="S3" t="n">
-        <v>1186.086815988008</v>
+        <v>1274.737295097263</v>
       </c>
       <c r="T3" t="n">
-        <v>22.47770596391397</v>
+        <v>16.68353608080734</v>
       </c>
       <c r="U3" t="n">
         <v>72</v>
@@ -691,13 +691,13 @@
         <v>51</v>
       </c>
       <c r="G4" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="H4" t="n">
         <v>33</v>
       </c>
       <c r="I4" t="n">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="J4" t="n">
         <v>37</v>
@@ -706,31 +706,31 @@
         <v>37</v>
       </c>
       <c r="L4" t="n">
-        <v>307.6642182652499</v>
+        <v>307.9295527404681</v>
       </c>
       <c r="M4" t="n">
-        <v>307.1724440172248</v>
+        <v>307.4463874385427</v>
       </c>
       <c r="N4" t="n">
-        <v>0.1598412226153141</v>
+        <v>0.1569077399766709</v>
       </c>
       <c r="O4" t="n">
-        <v>16.66188200256356</v>
+        <v>8.598435536609339</v>
       </c>
       <c r="P4" t="n">
-        <v>13.58179372510157</v>
+        <v>8.109582645222247</v>
       </c>
       <c r="Q4" t="n">
-        <v>18.48583657589275</v>
+        <v>5.685370196772603</v>
       </c>
       <c r="R4" t="n">
         <v>1757.282778271333</v>
       </c>
       <c r="S4" t="n">
-        <v>1247.140068614742</v>
+        <v>1376.006979243956</v>
       </c>
       <c r="T4" t="n">
-        <v>29.03020025942701</v>
+        <v>21.69689498706882</v>
       </c>
       <c r="U4" t="n">
         <v>78</v>
@@ -758,46 +758,46 @@
         <v>47</v>
       </c>
       <c r="G5" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="H5" t="n">
         <v>37</v>
       </c>
       <c r="I5" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="J5" t="n">
         <v>50</v>
       </c>
       <c r="K5" t="n">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="L5" t="n">
-        <v>342.5620574691616</v>
+        <v>345.1634236616073</v>
       </c>
       <c r="M5" t="n">
-        <v>341.7059296148391</v>
+        <v>342.4741617542422</v>
       </c>
       <c r="N5" t="n">
-        <v>0.2499190542722512</v>
+        <v>0.7791271389176972</v>
       </c>
       <c r="O5" t="n">
-        <v>30.83111887587454</v>
+        <v>15.8005324423661</v>
       </c>
       <c r="P5" t="n">
-        <v>26.3141666872662</v>
+        <v>13.26291140538589</v>
       </c>
       <c r="Q5" t="n">
-        <v>14.65062687732319</v>
+        <v>16.06035142319678</v>
       </c>
       <c r="R5" t="n">
         <v>5934.200144198503</v>
       </c>
       <c r="S5" t="n">
-        <v>3818.386020307053</v>
+        <v>3499.158634223997</v>
       </c>
       <c r="T5" t="n">
-        <v>35.65457976606923</v>
+        <v>41.0340307169298</v>
       </c>
       <c r="U5" t="n">
         <v>79</v>
@@ -837,34 +837,34 @@
         <v>63</v>
       </c>
       <c r="K6" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L6" t="n">
-        <v>373.8930567136795</v>
+        <v>384.0596934897975</v>
       </c>
       <c r="M6" t="n">
-        <v>369.7773865013562</v>
+        <v>369.9533072093814</v>
       </c>
       <c r="N6" t="n">
-        <v>1.100761337612902</v>
+        <v>3.672967124520935</v>
       </c>
       <c r="O6" t="n">
-        <v>36.63887170693729</v>
+        <v>23.60194337326843</v>
       </c>
       <c r="P6" t="n">
-        <v>20.8940869366643</v>
+        <v>10.72497314113647</v>
       </c>
       <c r="Q6" t="n">
-        <v>42.97289746313842</v>
+        <v>54.55894045876079</v>
       </c>
       <c r="R6" t="n">
         <v>6221.026445476135</v>
       </c>
       <c r="S6" t="n">
-        <v>2130.206872068994</v>
+        <v>2167.658954666326</v>
       </c>
       <c r="T6" t="n">
-        <v>65.75795183095455</v>
+        <v>65.15592766459585</v>
       </c>
       <c r="U6" t="n">
         <v>72</v>
@@ -907,22 +907,22 @@
         <v>37</v>
       </c>
       <c r="L7" t="n">
-        <v>655.3628625205121</v>
+        <v>681.673572754318</v>
       </c>
       <c r="M7" t="n">
-        <v>647.9281835230197</v>
+        <v>648.5257574718164</v>
       </c>
       <c r="N7" t="n">
-        <v>1.134437030639598</v>
+        <v>4.862710923142741</v>
       </c>
       <c r="O7" t="n">
-        <v>64.43067290305686</v>
+        <v>48.91290354276497</v>
       </c>
       <c r="P7" t="n">
-        <v>36.24326592986401</v>
+        <v>19.35823570212665</v>
       </c>
       <c r="Q7" t="n">
-        <v>43.74842866471991</v>
+        <v>60.42304933870552</v>
       </c>
       <c r="R7" t="n">
         <v>11589.41166652558</v>
@@ -971,34 +971,34 @@
         <v>85</v>
       </c>
       <c r="K8" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="L8" t="n">
-        <v>531.9747280589547</v>
+        <v>567.6061603149237</v>
       </c>
       <c r="M8" t="n">
-        <v>520.3269060646491</v>
+        <v>520.4966562161896</v>
       </c>
       <c r="N8" t="n">
-        <v>2.18954423583348</v>
+        <v>8.299681608916368</v>
       </c>
       <c r="O8" t="n">
-        <v>59.74227246612163</v>
+        <v>50.2027784940207</v>
       </c>
       <c r="P8" t="n">
-        <v>21.17585216415553</v>
+        <v>11.26208717459754</v>
       </c>
       <c r="Q8" t="n">
-        <v>64.55465905458512</v>
+        <v>77.5668050406037</v>
       </c>
       <c r="R8" t="n">
         <v>7364.606029970773</v>
       </c>
       <c r="S8" t="n">
-        <v>2411.443276119529</v>
+        <v>2236.729697787815</v>
       </c>
       <c r="T8" t="n">
-        <v>67.25631668135411</v>
+        <v>69.62865781706056</v>
       </c>
       <c r="U8" t="n">
         <v>76</v>
@@ -1026,46 +1026,46 @@
         <v>51</v>
       </c>
       <c r="G9" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H9" t="n">
         <v>33</v>
       </c>
       <c r="I9" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J9" t="n">
         <v>8</v>
       </c>
       <c r="K9" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="L9" t="n">
-        <v>569.798743281367</v>
+        <v>621.7350805802553</v>
       </c>
       <c r="M9" t="n">
-        <v>560.5421317098428</v>
+        <v>566.6366401697672</v>
       </c>
       <c r="N9" t="n">
-        <v>1.624540538334128</v>
+        <v>8.862044644330757</v>
       </c>
       <c r="O9" t="n">
-        <v>80.26733923816782</v>
+        <v>68.24623710845452</v>
       </c>
       <c r="P9" t="n">
-        <v>53.4891076946555</v>
+        <v>27.03636362145501</v>
       </c>
       <c r="Q9" t="n">
-        <v>33.36130460741501</v>
+        <v>60.38409622718133</v>
       </c>
       <c r="R9" t="n">
         <v>8564.572824595154</v>
       </c>
       <c r="S9" t="n">
-        <v>11143.33818026989</v>
+        <v>11375.92136920396</v>
       </c>
       <c r="T9" t="n">
-        <v>-30.10967865518305</v>
+        <v>-32.82532126453947</v>
       </c>
       <c r="U9" t="n">
         <v>57</v>
@@ -1093,46 +1093,46 @@
         <v>54</v>
       </c>
       <c r="G10" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H10" t="n">
         <v>30</v>
       </c>
       <c r="I10" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J10" t="n">
         <v>18</v>
       </c>
       <c r="K10" t="n">
-        <v>31</v>
+        <v>71</v>
       </c>
       <c r="L10" t="n">
-        <v>526.534714483452</v>
+        <v>540.2734330503725</v>
       </c>
       <c r="M10" t="n">
-        <v>520.4995410992019</v>
+        <v>520.6034882989749</v>
       </c>
       <c r="N10" t="n">
-        <v>1.146206169933322</v>
+        <v>3.640738845947242</v>
       </c>
       <c r="O10" t="n">
-        <v>42.66978385827319</v>
+        <v>29.36996351780499</v>
       </c>
       <c r="P10" t="n">
-        <v>19.7969643340029</v>
+        <v>11.34201644895668</v>
       </c>
       <c r="Q10" t="n">
-        <v>53.60425447722419</v>
+        <v>61.38225898006036</v>
       </c>
       <c r="R10" t="n">
         <v>8220.682866934612</v>
       </c>
       <c r="S10" t="n">
-        <v>2846.077115272143</v>
+        <v>2373.476981200878</v>
       </c>
       <c r="T10" t="n">
-        <v>65.37906690550382</v>
+        <v>71.12798267954695</v>
       </c>
       <c r="U10" t="n">
         <v>247</v>
@@ -1160,13 +1160,13 @@
         <v>49</v>
       </c>
       <c r="G11" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H11" t="n">
         <v>35</v>
       </c>
       <c r="I11" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="J11" t="n">
         <v>60</v>
@@ -1175,31 +1175,31 @@
         <v>60</v>
       </c>
       <c r="L11" t="n">
-        <v>882.4051599539741</v>
+        <v>1198.459124195285</v>
       </c>
       <c r="M11" t="n">
-        <v>882.3513868613016</v>
+        <v>1206.552808222636</v>
       </c>
       <c r="N11" t="n">
-        <v>0.006093923190033361</v>
+        <v>-0.6753408492580245</v>
       </c>
       <c r="O11" t="n">
-        <v>340.6405696868044</v>
+        <v>323.2067645892409</v>
       </c>
       <c r="P11" t="n">
-        <v>368.8582338411085</v>
+        <v>361.3220671409791</v>
       </c>
       <c r="Q11" t="n">
-        <v>-8.283706247981076</v>
+        <v>-11.79285421212593</v>
       </c>
       <c r="R11" t="n">
         <v>25546.30942574752</v>
       </c>
       <c r="S11" t="n">
-        <v>24427.45610376421</v>
+        <v>24524.39045338232</v>
       </c>
       <c r="T11" t="n">
-        <v>4.379706294701193</v>
+        <v>4.000260684759538</v>
       </c>
       <c r="U11" t="n">
         <v>346</v>
@@ -1227,46 +1227,46 @@
         <v>47</v>
       </c>
       <c r="G12" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H12" t="n">
         <v>37</v>
       </c>
       <c r="I12" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="J12" t="n">
         <v>29</v>
       </c>
       <c r="K12" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L12" t="n">
-        <v>600.4948874489901</v>
+        <v>637.2700861171445</v>
       </c>
       <c r="M12" t="n">
-        <v>596.7778850979574</v>
+        <v>608.9217866771495</v>
       </c>
       <c r="N12" t="n">
-        <v>0.6189898413328945</v>
+        <v>4.448396379739053</v>
       </c>
       <c r="O12" t="n">
-        <v>80.80844452480299</v>
+        <v>61.80059319701445</v>
       </c>
       <c r="P12" t="n">
-        <v>67.42980586311407</v>
+        <v>38.80375360735096</v>
       </c>
       <c r="Q12" t="n">
-        <v>16.55599082541744</v>
+        <v>37.21135736731805</v>
       </c>
       <c r="R12" t="n">
         <v>13337.49627232665</v>
       </c>
       <c r="S12" t="n">
-        <v>14573.88476163218</v>
+        <v>14879.75865451574</v>
       </c>
       <c r="T12" t="n">
-        <v>-9.270019380405436</v>
+        <v>-11.56335755001531</v>
       </c>
       <c r="U12" t="n">
         <v>133</v>
@@ -1306,34 +1306,34 @@
         <v>52</v>
       </c>
       <c r="K13" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="L13" t="n">
-        <v>514.2973437495663</v>
+        <v>578.1448337770589</v>
       </c>
       <c r="M13" t="n">
-        <v>501.1317243332446</v>
+        <v>506.5615504920752</v>
       </c>
       <c r="N13" t="n">
-        <v>2.559923666013063</v>
+        <v>12.38154855026989</v>
       </c>
       <c r="O13" t="n">
-        <v>91.30817694719278</v>
+        <v>80.17019778833863</v>
       </c>
       <c r="P13" t="n">
-        <v>53.20084278119364</v>
+        <v>27.101376225873</v>
       </c>
       <c r="Q13" t="n">
-        <v>41.73485381056086</v>
+        <v>66.19519849829395</v>
       </c>
       <c r="R13" t="n">
         <v>9020.125377233937</v>
       </c>
       <c r="S13" t="n">
-        <v>11834.55910827189</v>
+        <v>12214.04556241399</v>
       </c>
       <c r="T13" t="n">
-        <v>-31.20171409303634</v>
+        <v>-35.40882251194917</v>
       </c>
       <c r="U13" t="n">
         <v>53</v>
@@ -1361,46 +1361,46 @@
         <v>60</v>
       </c>
       <c r="G14" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H14" t="n">
         <v>24</v>
       </c>
       <c r="I14" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="J14" t="n">
         <v>61</v>
       </c>
       <c r="K14" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L14" t="n">
-        <v>970.0898978633646</v>
+        <v>1640.523312738835</v>
       </c>
       <c r="M14" t="n">
-        <v>884.7612059752666</v>
+        <v>1291.294291498908</v>
       </c>
       <c r="N14" t="n">
-        <v>8.795957166035386</v>
+        <v>21.28765976857065</v>
       </c>
       <c r="O14" t="n">
-        <v>424.3554447984706</v>
+        <v>405.2496962111079</v>
       </c>
       <c r="P14" t="n">
-        <v>423.2500150517187</v>
+        <v>415.3955108567552</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.2604961855212709</v>
+        <v>-2.503595867068094</v>
       </c>
       <c r="R14" t="n">
         <v>25608.69285909054</v>
       </c>
       <c r="S14" t="n">
-        <v>24591.70443437644</v>
+        <v>23868.64892963442</v>
       </c>
       <c r="T14" t="n">
-        <v>3.971262533039048</v>
+        <v>6.794739345075359</v>
       </c>
       <c r="U14" t="n">
         <v>173</v>
@@ -1428,46 +1428,46 @@
         <v>60</v>
       </c>
       <c r="G15" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H15" t="n">
         <v>24</v>
       </c>
       <c r="I15" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="L15" t="n">
-        <v>513.9030635117903</v>
+        <v>674.4537163265511</v>
       </c>
       <c r="M15" t="n">
-        <v>472.2290618001111</v>
+        <v>480.8462316820936</v>
       </c>
       <c r="N15" t="n">
-        <v>8.10931178866635</v>
+        <v>28.70582220214476</v>
       </c>
       <c r="O15" t="n">
-        <v>140.4832910838326</v>
+        <v>133.8196132819058</v>
       </c>
       <c r="P15" t="n">
-        <v>58.70499365515283</v>
+        <v>30.92676778176923</v>
       </c>
       <c r="Q15" t="n">
-        <v>58.21211675620487</v>
+        <v>76.88921151145568</v>
       </c>
       <c r="R15" t="n">
         <v>9001.20224906488</v>
       </c>
       <c r="S15" t="n">
-        <v>11092.64231706538</v>
+        <v>11741.85464429577</v>
       </c>
       <c r="T15" t="n">
-        <v>-23.23511915553028</v>
+        <v>-30.44762598813519</v>
       </c>
       <c r="U15" t="n">
         <v>94</v>
@@ -1507,34 +1507,34 @@
         <v>16</v>
       </c>
       <c r="K16" t="n">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="L16" t="n">
-        <v>534.197975363023</v>
+        <v>568.6735765878643</v>
       </c>
       <c r="M16" t="n">
-        <v>525.7558967126967</v>
+        <v>527.0496423444907</v>
       </c>
       <c r="N16" t="n">
-        <v>1.580327713632652</v>
+        <v>7.319477457195054</v>
       </c>
       <c r="O16" t="n">
-        <v>65.03350811650294</v>
+        <v>52.55351123541791</v>
       </c>
       <c r="P16" t="n">
-        <v>36.53680690747105</v>
+        <v>17.86371621572818</v>
       </c>
       <c r="Q16" t="n">
-        <v>43.81848993596049</v>
+        <v>66.0085200859251</v>
       </c>
       <c r="R16" t="n">
         <v>8602.635858334566</v>
       </c>
       <c r="S16" t="n">
-        <v>5972.637880757733</v>
+        <v>5736.654365469741</v>
       </c>
       <c r="T16" t="n">
-        <v>30.57200166189517</v>
+        <v>33.31515526242055</v>
       </c>
       <c r="U16" t="n">
         <v>80</v>
@@ -1574,34 +1574,34 @@
         <v>30</v>
       </c>
       <c r="K17" t="n">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="L17" t="n">
-        <v>405.3822220764889</v>
+        <v>412.8920981560133</v>
       </c>
       <c r="M17" t="n">
-        <v>402.5854832001096</v>
+        <v>403.0697803347077</v>
       </c>
       <c r="N17" t="n">
-        <v>0.6899017085785336</v>
+        <v>2.378906708356074</v>
       </c>
       <c r="O17" t="n">
-        <v>38.55796762786584</v>
+        <v>22.94273561661126</v>
       </c>
       <c r="P17" t="n">
-        <v>27.36279122650203</v>
+        <v>13.87291781898569</v>
       </c>
       <c r="Q17" t="n">
-        <v>29.03466414363876</v>
+        <v>39.53241648767785</v>
       </c>
       <c r="R17" t="n">
         <v>6932.210741623266</v>
       </c>
       <c r="S17" t="n">
-        <v>3980.636011170929</v>
+        <v>3482.577171215869</v>
       </c>
       <c r="T17" t="n">
-        <v>42.57768323069168</v>
+        <v>49.76238748332716</v>
       </c>
       <c r="U17" t="n">
         <v>80</v>
@@ -1641,34 +1641,34 @@
         <v>44</v>
       </c>
       <c r="K18" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="L18" t="n">
-        <v>505.7162503342355</v>
+        <v>637.0069727381103</v>
       </c>
       <c r="M18" t="n">
-        <v>479.1292433443459</v>
+        <v>506.6342629503388</v>
       </c>
       <c r="N18" t="n">
-        <v>5.257297342594365</v>
+        <v>20.46644940594254</v>
       </c>
       <c r="O18" t="n">
-        <v>132.517794650461</v>
+        <v>123.5598598374653</v>
       </c>
       <c r="P18" t="n">
-        <v>80.78355847789373</v>
+        <v>54.51580243051097</v>
       </c>
       <c r="Q18" t="n">
-        <v>39.0394635747036</v>
+        <v>55.87903506670951</v>
       </c>
       <c r="R18" t="n">
         <v>7583.043852209177</v>
       </c>
       <c r="S18" t="n">
-        <v>12205.50650031101</v>
+        <v>12254.18537071123</v>
       </c>
       <c r="T18" t="n">
-        <v>-60.95787836905578</v>
+        <v>-61.59982204429954</v>
       </c>
       <c r="U18" t="n">
         <v>73</v>
@@ -1711,22 +1711,22 @@
         <v>68</v>
       </c>
       <c r="L19" t="n">
-        <v>1013.358576203901</v>
+        <v>1124.831094818783</v>
       </c>
       <c r="M19" t="n">
-        <v>996.3773294534783</v>
+        <v>1032.288936677678</v>
       </c>
       <c r="N19" t="n">
-        <v>1.675739185435792</v>
+        <v>8.227204828118069</v>
       </c>
       <c r="O19" t="n">
-        <v>137.1045077958579</v>
+        <v>124.8091969639001</v>
       </c>
       <c r="P19" t="n">
-        <v>98.73532622198965</v>
+        <v>69.51630022491672</v>
       </c>
       <c r="Q19" t="n">
-        <v>27.98535379376305</v>
+        <v>44.30194094989359</v>
       </c>
       <c r="R19" t="n">
         <v>11378.44495796659</v>
@@ -1763,46 +1763,46 @@
         <v>52</v>
       </c>
       <c r="G20" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H20" t="n">
         <v>32</v>
       </c>
       <c r="I20" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J20" t="n">
         <v>69</v>
       </c>
       <c r="K20" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="L20" t="n">
-        <v>312.7896037366755</v>
+        <v>320.2185116188592</v>
       </c>
       <c r="M20" t="n">
-        <v>309.2115266907489</v>
+        <v>309.3654127486924</v>
       </c>
       <c r="N20" t="n">
-        <v>1.143924543265455</v>
+        <v>3.38927903177712</v>
       </c>
       <c r="O20" t="n">
-        <v>33.30213553364789</v>
+        <v>20.1682285568437</v>
       </c>
       <c r="P20" t="n">
-        <v>19.56204275646797</v>
+        <v>10.1235026574799</v>
       </c>
       <c r="Q20" t="n">
-        <v>41.25889393278451</v>
+        <v>49.80470084942245</v>
       </c>
       <c r="R20" t="n">
         <v>6289.823265409355</v>
       </c>
       <c r="S20" t="n">
-        <v>2160.136483810634</v>
+        <v>2114.530977438321</v>
       </c>
       <c r="T20" t="n">
-        <v>65.6566426009102</v>
+        <v>66.38171076972698</v>
       </c>
       <c r="U20" t="n">
         <v>77</v>
@@ -1842,34 +1842,34 @@
         <v>82</v>
       </c>
       <c r="K21" t="n">
-        <v>51</v>
+        <v>82</v>
       </c>
       <c r="L21" t="n">
-        <v>341.819816871587</v>
+        <v>347.7946633940018</v>
       </c>
       <c r="M21" t="n">
-        <v>337.9161716024215</v>
+        <v>337.9557111041366</v>
       </c>
       <c r="N21" t="n">
-        <v>1.142018419204762</v>
+        <v>2.828954358830717</v>
       </c>
       <c r="O21" t="n">
-        <v>30.36945124682518</v>
+        <v>17.89907040534108</v>
       </c>
       <c r="P21" t="n">
-        <v>15.10104121215474</v>
+        <v>8.641522555143561</v>
       </c>
       <c r="Q21" t="n">
-        <v>50.27555457152555</v>
+        <v>51.72083041494193</v>
       </c>
       <c r="R21" t="n">
         <v>6489.895548146145</v>
       </c>
       <c r="S21" t="n">
-        <v>1773.280205030827</v>
+        <v>1895.480866864503</v>
       </c>
       <c r="T21" t="n">
-        <v>72.67629052154207</v>
+        <v>70.79335325503116</v>
       </c>
       <c r="U21" t="n">
         <v>52</v>
@@ -1909,34 +1909,34 @@
         <v>1</v>
       </c>
       <c r="K22" t="n">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="L22" t="n">
-        <v>340.8106425229002</v>
+        <v>432.2414306693133</v>
       </c>
       <c r="M22" t="n">
-        <v>314.1572968940865</v>
+        <v>315.068420395681</v>
       </c>
       <c r="N22" t="n">
-        <v>7.820573158017739</v>
+        <v>27.10823210357075</v>
       </c>
       <c r="O22" t="n">
-        <v>103.3591846743154</v>
+        <v>96.11927017659771</v>
       </c>
       <c r="P22" t="n">
-        <v>31.91639883809943</v>
+        <v>15.87685244616273</v>
       </c>
       <c r="Q22" t="n">
-        <v>69.1208875740768</v>
+        <v>83.48213379378292</v>
       </c>
       <c r="R22" t="n">
         <v>8122.751979971314</v>
       </c>
       <c r="S22" t="n">
-        <v>4776.695432049399</v>
+        <v>4551.418795848092</v>
       </c>
       <c r="T22" t="n">
-        <v>41.1936318648219</v>
+        <v>43.96703473070753</v>
       </c>
       <c r="U22" t="n">
         <v>56</v>
@@ -1964,13 +1964,13 @@
         <v>51</v>
       </c>
       <c r="G23" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H23" t="n">
         <v>33</v>
       </c>
       <c r="I23" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="J23" t="n">
         <v>10</v>
@@ -1979,31 +1979,31 @@
         <v>89</v>
       </c>
       <c r="L23" t="n">
-        <v>439.546099357842</v>
+        <v>541.4702005763756</v>
       </c>
       <c r="M23" t="n">
-        <v>430.6775879000923</v>
+        <v>498.6589038026857</v>
       </c>
       <c r="N23" t="n">
-        <v>2.017652180443912</v>
+        <v>7.90649175672435</v>
       </c>
       <c r="O23" t="n">
-        <v>127.6021684603201</v>
+        <v>111.9918718762339</v>
       </c>
       <c r="P23" t="n">
-        <v>116.8400585680568</v>
+        <v>98.90909911374817</v>
       </c>
       <c r="Q23" t="n">
-        <v>8.43411207044649</v>
+        <v>11.68189489407225</v>
       </c>
       <c r="R23" t="n">
         <v>10981.77096754267</v>
       </c>
       <c r="S23" t="n">
-        <v>12706.65305839169</v>
+        <v>12757.07628481388</v>
       </c>
       <c r="T23" t="n">
-        <v>-15.70677530925585</v>
+        <v>-16.16592917953069</v>
       </c>
       <c r="U23" t="n">
         <v>193</v>
@@ -2046,22 +2046,22 @@
         <v>69</v>
       </c>
       <c r="L24" t="n">
-        <v>822.2578227067829</v>
+        <v>1225.299688363582</v>
       </c>
       <c r="M24" t="n">
-        <v>789.6866432584886</v>
+        <v>1096.759844798069</v>
       </c>
       <c r="N24" t="n">
-        <v>3.961188151554889</v>
+        <v>10.49048202543668</v>
       </c>
       <c r="O24" t="n">
-        <v>343.0985870950429</v>
+        <v>319.4976124798335</v>
       </c>
       <c r="P24" t="n">
-        <v>355.8910862374291</v>
+        <v>341.9565867427467</v>
       </c>
       <c r="Q24" t="n">
-        <v>-3.728519913386439</v>
+        <v>-7.029465443761591</v>
       </c>
       <c r="R24" t="n">
         <v>27841.51805172316</v>
@@ -2098,46 +2098,46 @@
         <v>47</v>
       </c>
       <c r="G25" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H25" t="n">
         <v>37</v>
       </c>
       <c r="I25" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J25" t="n">
         <v>70</v>
       </c>
       <c r="K25" t="n">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="L25" t="n">
-        <v>478.2294827164522</v>
+        <v>509.3885635883431</v>
       </c>
       <c r="M25" t="n">
-        <v>475.0091036960562</v>
+        <v>481.4975047857588</v>
       </c>
       <c r="N25" t="n">
-        <v>0.6733961699942753</v>
+        <v>5.475399487987745</v>
       </c>
       <c r="O25" t="n">
-        <v>74.14480912028561</v>
+        <v>55.36262259877862</v>
       </c>
       <c r="P25" t="n">
-        <v>61.98526724990769</v>
+        <v>31.87026250979933</v>
       </c>
       <c r="Q25" t="n">
-        <v>16.39972105215272</v>
+        <v>42.43361131793198</v>
       </c>
       <c r="R25" t="n">
         <v>9575.213752498366</v>
       </c>
       <c r="S25" t="n">
-        <v>14683.87043596455</v>
+        <v>14681.92431192803</v>
       </c>
       <c r="T25" t="n">
-        <v>-53.35292574678277</v>
+        <v>-53.33260114529783</v>
       </c>
       <c r="U25" t="n">
         <v>167</v>
@@ -2165,46 +2165,46 @@
         <v>47</v>
       </c>
       <c r="G26" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H26" t="n">
         <v>37</v>
       </c>
       <c r="I26" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="J26" t="n">
         <v>8</v>
       </c>
       <c r="K26" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="L26" t="n">
-        <v>385.7045371017182</v>
+        <v>416.9957713136897</v>
       </c>
       <c r="M26" t="n">
-        <v>383.296273319798</v>
+        <v>396.962930104445</v>
       </c>
       <c r="N26" t="n">
-        <v>0.6243804649062327</v>
+        <v>4.804087376266149</v>
       </c>
       <c r="O26" t="n">
-        <v>70.15568087631378</v>
+        <v>52.01916346956003</v>
       </c>
       <c r="P26" t="n">
-        <v>62.00397429228353</v>
+        <v>36.62764231577655</v>
       </c>
       <c r="Q26" t="n">
-        <v>11.6194533104196</v>
+        <v>29.58817506319591</v>
       </c>
       <c r="R26" t="n">
         <v>8440.722109454817</v>
       </c>
       <c r="S26" t="n">
-        <v>11388.90103452508</v>
+        <v>11242.32561037166</v>
       </c>
       <c r="T26" t="n">
-        <v>-34.92804154478535</v>
+        <v>-33.1915144769267</v>
       </c>
       <c r="U26" t="n">
         <v>204</v>
@@ -2244,34 +2244,34 @@
         <v>43</v>
       </c>
       <c r="K27" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="L27" t="n">
-        <v>469.4623174552167</v>
+        <v>567.5142341339715</v>
       </c>
       <c r="M27" t="n">
-        <v>464.5800101651473</v>
+        <v>540.8398293915541</v>
       </c>
       <c r="N27" t="n">
-        <v>1.039978526186006</v>
+        <v>4.700217745749172</v>
       </c>
       <c r="O27" t="n">
-        <v>129.4405324776689</v>
+        <v>111.434856830445</v>
       </c>
       <c r="P27" t="n">
-        <v>128.594872359449</v>
+        <v>108.7007641663532</v>
       </c>
       <c r="Q27" t="n">
-        <v>0.6533194062422264</v>
+        <v>2.45353450604052</v>
       </c>
       <c r="R27" t="n">
         <v>15191.6961406471</v>
       </c>
       <c r="S27" t="n">
-        <v>12906.83876641361</v>
+        <v>13109.47572504328</v>
       </c>
       <c r="T27" t="n">
-        <v>15.04017295422394</v>
+        <v>13.70630636846799</v>
       </c>
       <c r="U27" t="n">
         <v>9999</v>
@@ -2342,7 +2342,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>63</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6">
@@ -2362,7 +2362,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>70.95999999999999</v>
+        <v>168.31</v>
       </c>
     </row>
     <row r="8">
@@ -2372,7 +2372,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5.49</v>
+        <v>14.63</v>
       </c>
     </row>
     <row r="9">
@@ -2382,7 +2382,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>79.81999999999999</v>
+        <v>187.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>